<commit_message>
feat(comm): Komunikasi jadi kotak masuk pribadi utk Leader + notifikasi hilang saat dibaca
</commit_message>
<xml_diff>
--- a/gas/data-dummy/ProductTrack-Data-Dummy.xlsx
+++ b/gas/data-dummy/ProductTrack-Data-Dummy.xlsx
@@ -237,10 +237,10 @@
         </is>
       </c>
       <c r="C4" s="1">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="D4" s="1">
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
@@ -313,10 +313,10 @@
         </is>
       </c>
       <c r="C5" s="1">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="D5" s="1">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
@@ -399,10 +399,10 @@
         </is>
       </c>
       <c r="C6" s="1">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="D6" s="1">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
@@ -475,10 +475,10 @@
         </is>
       </c>
       <c r="C7" s="1">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="D7" s="1">
-        <v>46200</v>
+        <v>46201</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="C8" s="1">
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="D8" s="1">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
@@ -632,10 +632,10 @@
         </is>
       </c>
       <c r="C9" s="1">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="D9" s="1">
-        <v>46205</v>
+        <v>46206</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="C10" s="1">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="D10" s="1">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
@@ -784,10 +784,10 @@
         </is>
       </c>
       <c r="C11" s="1">
-        <v>46200</v>
+        <v>46201</v>
       </c>
       <c r="D11" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
@@ -860,10 +860,10 @@
         </is>
       </c>
       <c r="C12" s="1">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="D12" s="1">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
@@ -913,10 +913,10 @@
         </is>
       </c>
       <c r="C13" s="1">
-        <v>46205</v>
+        <v>46206</v>
       </c>
       <c r="D13" s="1">
-        <v>46215</v>
+        <v>46216</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
@@ -994,10 +994,10 @@
         </is>
       </c>
       <c r="C14" s="1">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D14" s="1">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="C15" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D15" s="1">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
@@ -1136,10 +1136,10 @@
         </is>
       </c>
       <c r="C16" s="1">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="D16" s="1">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="C17" s="1">
-        <v>46215</v>
+        <v>46216</v>
       </c>
       <c r="D17" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
@@ -1293,10 +1293,10 @@
         </is>
       </c>
       <c r="C18" s="1">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="D18" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -1379,10 +1379,10 @@
         </is>
       </c>
       <c r="C19" s="1">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D19" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
@@ -1450,10 +1450,10 @@
         </is>
       </c>
       <c r="C20" s="1">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D20" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
@@ -1531,10 +1531,10 @@
         </is>
       </c>
       <c r="C21" s="1">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="D21" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         </is>
       </c>
       <c r="C22" s="1">
-        <v>46215</v>
+        <v>46216</v>
       </c>
       <c r="D22" s="1">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -1703,10 +1703,10 @@
         </is>
       </c>
       <c r="C23" s="1">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="D23" s="1">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -1769,10 +1769,10 @@
         </is>
       </c>
       <c r="C24" s="1">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="D24" s="1">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -1845,10 +1845,10 @@
         </is>
       </c>
       <c r="C25" s="1">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="D25" s="1">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -1931,10 +1931,10 @@
         </is>
       </c>
       <c r="C26" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="D26" s="1">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -2002,10 +2002,10 @@
         </is>
       </c>
       <c r="C27" s="1">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="D27" s="1">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -2083,10 +2083,10 @@
         </is>
       </c>
       <c r="C28" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="D28" s="1">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
@@ -2149,10 +2149,10 @@
         </is>
       </c>
       <c r="C29" s="1">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="D29" s="1">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -2225,10 +2225,10 @@
         </is>
       </c>
       <c r="C30" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="D30" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -2296,10 +2296,10 @@
         </is>
       </c>
       <c r="C31" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="D31" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
@@ -2362,10 +2362,10 @@
         </is>
       </c>
       <c r="C32" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="D32" s="1">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
@@ -2428,10 +2428,10 @@
         </is>
       </c>
       <c r="C33" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="D33" s="1">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
@@ -2494,10 +2494,10 @@
         </is>
       </c>
       <c r="C34" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="D34" s="1">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
@@ -2560,10 +2560,10 @@
         </is>
       </c>
       <c r="C35" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="D35" s="1">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
@@ -2626,10 +2626,10 @@
         </is>
       </c>
       <c r="C36" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="D36" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
@@ -2702,10 +2702,10 @@
         </is>
       </c>
       <c r="C37" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="D37" s="1">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
@@ -2773,10 +2773,10 @@
         </is>
       </c>
       <c r="C38" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="D38" s="1">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
@@ -2844,10 +2844,10 @@
         </is>
       </c>
       <c r="C39" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="D39" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
@@ -2910,10 +2910,10 @@
         </is>
       </c>
       <c r="C40" s="1">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="D40" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
@@ -2968,10 +2968,10 @@
         </is>
       </c>
       <c r="C41" s="1">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="D41" s="1">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
@@ -3026,10 +3026,10 @@
         </is>
       </c>
       <c r="C42" s="1">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="D42" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
@@ -3079,10 +3079,10 @@
         </is>
       </c>
       <c r="C43" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="D43" s="1">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
@@ -3127,10 +3127,10 @@
         </is>
       </c>
       <c r="C44" s="1">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="D44" s="1">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
@@ -3185,10 +3185,10 @@
         </is>
       </c>
       <c r="C45" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="D45" s="1">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
@@ -3233,10 +3233,10 @@
         </is>
       </c>
       <c r="C46" s="1">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="D46" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
@@ -3286,10 +3286,10 @@
         </is>
       </c>
       <c r="C47" s="1">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="D47" s="1">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
@@ -3339,10 +3339,10 @@
         </is>
       </c>
       <c r="C48" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="D48" s="1">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
@@ -3392,10 +3392,10 @@
         </is>
       </c>
       <c r="C49" s="1">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D49" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
@@ -3455,10 +3455,10 @@
         </is>
       </c>
       <c r="C50" s="1">
-        <v>46214</v>
+        <v>46215</v>
       </c>
       <c r="D50" s="1">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         </is>
       </c>
       <c r="C51" s="1">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="D51" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
@@ -3581,10 +3581,10 @@
         </is>
       </c>
       <c r="C52" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="D52" s="1">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
@@ -3644,59 +3644,319 @@
         </is>
       </c>
       <c r="C53" s="1">
+        <v>46229</v>
+      </c>
+      <c r="D53" s="1">
+        <v>46242</v>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review PM</t>
+        </is>
+      </c>
+      <c r="F53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Normal</t>
+        </is>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request data closing penjualan Juli</t>
+        </is>
+      </c>
+      <c r="H53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data &amp; Intelligence</t>
+        </is>
+      </c>
+      <c r="I53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All Platform</t>
+        </is>
+      </c>
+      <c r="J53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff Data</t>
+        </is>
+      </c>
+      <c r="M53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data sudah dikirim, menunggu konfirmasi.</t>
+        </is>
+      </c>
+      <c r="O53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sales</t>
+        </is>
+      </c>
+      <c r="P53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kontak Sales</t>
+        </is>
+      </c>
+      <c r="U53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TSK-051</t>
+        </is>
+      </c>
+      <c r="C54" s="1">
+        <v>46225</v>
+      </c>
+      <c r="D54" s="1">
+        <v>46233</v>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review PM</t>
+        </is>
+      </c>
+      <c r="F54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Normal</t>
+        </is>
+      </c>
+      <c r="G54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Merapikan 40 soal hasil input magang</t>
+        </is>
+      </c>
+      <c r="H54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC Konten</t>
+        </is>
+      </c>
+      <c r="I54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JadiASN</t>
+        </is>
+      </c>
+      <c r="J54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magang Konten</t>
+        </is>
+      </c>
+      <c r="K54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff QC</t>
+        </is>
+      </c>
+      <c r="L54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Latihan Batch 1</t>
+        </is>
+      </c>
+      <c r="M54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sudah selesai, mohon direview.</t>
+        </is>
+      </c>
+      <c r="N54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cek konsistensi format.</t>
+        </is>
+      </c>
+      <c r="U54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff QC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TSK-052</t>
+        </is>
+      </c>
+      <c r="C55" s="1">
         <v>46228</v>
       </c>
-      <c r="D53" s="1">
-        <v>46241</v>
-      </c>
-      <c r="E53" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review PM</t>
-        </is>
-      </c>
-      <c r="F53" s="0" t="inlineStr">
+      <c r="D55" s="1">
+        <v>46236</v>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In progress</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Normal</t>
         </is>
       </c>
-      <c r="G53" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Request data closing penjualan Juli</t>
-        </is>
-      </c>
-      <c r="H53" s="0" t="inlineStr">
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Menginput 60 soal latihan ke SIADU</t>
+        </is>
+      </c>
+      <c r="H55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input</t>
+        </is>
+      </c>
+      <c r="I55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Siadu</t>
+        </is>
+      </c>
+      <c r="J55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magang Konten</t>
+        </is>
+      </c>
+      <c r="K55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff Input</t>
+        </is>
+      </c>
+      <c r="M55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35 dari 60 selesai.</t>
+        </is>
+      </c>
+      <c r="Q55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Menginput</t>
+        </is>
+      </c>
+      <c r="R55" s="0">
+        <v>60</v>
+      </c>
+      <c r="S55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soal</t>
+        </is>
+      </c>
+      <c r="T55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">latihan magang</t>
+        </is>
+      </c>
+      <c r="U55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff Input</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TSK-053</t>
+        </is>
+      </c>
+      <c r="C56" s="1">
+        <v>46230</v>
+      </c>
+      <c r="D56" s="1">
+        <v>46234</v>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Todo</t>
+        </is>
+      </c>
+      <c r="F56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rekap data pendaftar mingguan</t>
+        </is>
+      </c>
+      <c r="H56" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Data &amp; Intelligence</t>
         </is>
       </c>
-      <c r="I53" s="0" t="inlineStr">
+      <c r="I56" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">All Platform</t>
         </is>
       </c>
-      <c r="J53" s="0" t="inlineStr">
+      <c r="J56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magang Data</t>
+        </is>
+      </c>
+      <c r="K56" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Staff Data</t>
         </is>
       </c>
-      <c r="M53" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data sudah dikirim, menunggu konfirmasi.</t>
-        </is>
-      </c>
-      <c r="O53" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sales</t>
-        </is>
-      </c>
-      <c r="P53" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kontak Sales</t>
-        </is>
-      </c>
-      <c r="U53" s="0" t="inlineStr">
+      <c r="N56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pakai template yang sudah ada.</t>
+        </is>
+      </c>
+      <c r="U56" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Staff Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TSK-054</t>
+        </is>
+      </c>
+      <c r="C57" s="1">
+        <v>46231</v>
+      </c>
+      <c r="D57" s="1">
+        <v>46240</v>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In progress</t>
+        </is>
+      </c>
+      <c r="F57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Belajar alur QC video pembahasan</t>
+        </is>
+      </c>
+      <c r="H57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC Konten</t>
+        </is>
+      </c>
+      <c r="I57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerebrum</t>
+        </is>
+      </c>
+      <c r="J57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magang Data</t>
+        </is>
+      </c>
+      <c r="L57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panduan Onboarding</t>
+        </is>
+      </c>
+      <c r="M57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedang mempelajari panduan.</t>
+        </is>
+      </c>
+      <c r="U57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff QC</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4453,7 @@
         </is>
       </c>
       <c r="D2" s="2">
-        <v>46231.583333333336</v>
+        <v>46232.583333333336</v>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
@@ -4218,7 +4478,7 @@
         </is>
       </c>
       <c r="D3" s="2">
-        <v>46225.583333333336</v>
+        <v>46226.583333333336</v>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
@@ -4243,7 +4503,7 @@
         </is>
       </c>
       <c r="D4" s="2">
-        <v>46229.583333333336</v>
+        <v>46230.583333333336</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
@@ -4268,7 +4528,7 @@
         </is>
       </c>
       <c r="D5" s="2">
-        <v>46221.583333333336</v>
+        <v>46222.583333333336</v>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
@@ -4293,7 +4553,7 @@
         </is>
       </c>
       <c r="D6" s="2">
-        <v>46227.583333333336</v>
+        <v>46228.583333333336</v>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
@@ -4318,7 +4578,7 @@
         </is>
       </c>
       <c r="D7" s="2">
-        <v>46232.583333333336</v>
+        <v>46233.583333333336</v>
       </c>
     </row>
     <row r="8">
@@ -4338,7 +4598,7 @@
         </is>
       </c>
       <c r="D8" s="2">
-        <v>46223.583333333336</v>
+        <v>46224.583333333336</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
@@ -4363,7 +4623,7 @@
         </is>
       </c>
       <c r="D9" s="2">
-        <v>46228.583333333336</v>
+        <v>46229.583333333336</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
@@ -4388,7 +4648,7 @@
         </is>
       </c>
       <c r="D10" s="2">
-        <v>46230.583333333336</v>
+        <v>46231.583333333336</v>
       </c>
     </row>
   </sheetData>
@@ -5139,7 +5399,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lintas Divisi</t>
+          <t xml:space="preserve">Magang Konten</t>
         </is>
       </c>
       <c r="C49" s="0" t="b">
@@ -5149,12 +5409,12 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">support</t>
+          <t xml:space="preserve">pic</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manager</t>
+          <t xml:space="preserve">Magang Data</t>
         </is>
       </c>
       <c r="C50" s="0" t="b">
@@ -5164,12 +5424,12 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">support</t>
+          <t xml:space="preserve">pic</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Soal</t>
+          <t xml:space="preserve">Lintas Divisi</t>
         </is>
       </c>
       <c r="C51" s="0" t="b">
@@ -5184,7 +5444,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leader Konten</t>
+          <t xml:space="preserve">Manager</t>
         </is>
       </c>
       <c r="C52" s="0" t="b">
@@ -5199,7 +5459,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Input</t>
+          <t xml:space="preserve">Staff Soal</t>
         </is>
       </c>
       <c r="C53" s="0" t="b">
@@ -5214,7 +5474,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leader Sistem</t>
+          <t xml:space="preserve">Leader Konten</t>
         </is>
       </c>
       <c r="C54" s="0" t="b">
@@ -5229,7 +5489,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Data</t>
+          <t xml:space="preserve">Staff Input</t>
         </is>
       </c>
       <c r="C55" s="0" t="b">
@@ -5244,7 +5504,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Materi</t>
+          <t xml:space="preserve">Leader Sistem</t>
         </is>
       </c>
       <c r="C56" s="0" t="b">
@@ -5259,7 +5519,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff QC</t>
+          <t xml:space="preserve">Staff Data</t>
         </is>
       </c>
       <c r="C57" s="0" t="b">
@@ -5274,7 +5534,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff Liveclass</t>
+          <t xml:space="preserve">Staff Materi</t>
         </is>
       </c>
       <c r="C58" s="0" t="b">
@@ -5289,7 +5549,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lintas Divisi</t>
+          <t xml:space="preserve">Staff QC</t>
         </is>
       </c>
       <c r="C59" s="0" t="b">
@@ -5299,12 +5559,12 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">division</t>
+          <t xml:space="preserve">support</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">IT</t>
+          <t xml:space="preserve">Staff Liveclass</t>
         </is>
       </c>
       <c r="C60" s="0" t="b">
@@ -5314,12 +5574,12 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">division</t>
+          <t xml:space="preserve">support</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marketing</t>
+          <t xml:space="preserve">Magang Konten</t>
         </is>
       </c>
       <c r="C61" s="0" t="b">
@@ -5329,12 +5589,12 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">division</t>
+          <t xml:space="preserve">support</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales</t>
+          <t xml:space="preserve">Magang Data</t>
         </is>
       </c>
       <c r="C62" s="0" t="b">
@@ -5344,92 +5604,72 @@
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">support</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menyusun</t>
+          <t xml:space="preserve">Lintas Divisi</t>
         </is>
       </c>
       <c r="C63" s="0" t="b">
         <v>1</v>
-      </c>
-      <c r="D63" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RnD</t>
-        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">division</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">kurikulum</t>
+          <t xml:space="preserve">IT</t>
         </is>
       </c>
       <c r="C64" s="0" t="b">
         <v>1</v>
-      </c>
-      <c r="D64" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RnD||Menyusun</t>
-        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">division</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">product knowledge</t>
+          <t xml:space="preserve">Marketing</t>
         </is>
       </c>
       <c r="C65" s="0" t="b">
         <v>1</v>
-      </c>
-      <c r="D65" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RnD||Menyusun</t>
-        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">division</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">silabus</t>
+          <t xml:space="preserve">Sales</t>
         </is>
       </c>
       <c r="C66" s="0" t="b">
         <v>1</v>
-      </c>
-      <c r="D66" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RnD||Menyusun</t>
-        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">sistem penilaian</t>
+          <t xml:space="preserve">Menyusun</t>
         </is>
       </c>
       <c r="C67" s="0" t="b">
@@ -5437,7 +5677,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RnD||Menyusun</t>
+          <t xml:space="preserve">RnD</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5689,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">panduan</t>
+          <t xml:space="preserve">kurikulum</t>
         </is>
       </c>
       <c r="C68" s="0" t="b">
@@ -5464,12 +5704,12 @@
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membuat</t>
+          <t xml:space="preserve">product knowledge</t>
         </is>
       </c>
       <c r="C69" s="0" t="b">
@@ -5477,7 +5717,7 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RnD</t>
+          <t xml:space="preserve">RnD||Menyusun</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5729,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapping</t>
+          <t xml:space="preserve">silabus</t>
         </is>
       </c>
       <c r="C70" s="0" t="b">
@@ -5497,7 +5737,7 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RnD||Membuat</t>
+          <t xml:space="preserve">RnD||Menyusun</t>
         </is>
       </c>
     </row>
@@ -5509,7 +5749,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">prompt</t>
+          <t xml:space="preserve">sistem penilaian</t>
         </is>
       </c>
       <c r="C71" s="0" t="b">
@@ -5517,19 +5757,19 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RnD||Membuat</t>
+          <t xml:space="preserve">RnD||Menyusun</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Melakukan</t>
+          <t xml:space="preserve">panduan</t>
         </is>
       </c>
       <c r="C72" s="0" t="b">
@@ -5537,19 +5777,19 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RnD</t>
+          <t xml:space="preserve">RnD||Menyusun</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">riset</t>
+          <t xml:space="preserve">Membuat</t>
         </is>
       </c>
       <c r="C73" s="0" t="b">
@@ -5557,19 +5797,19 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RnD||Melakukan</t>
+          <t xml:space="preserve">RnD</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menyusun</t>
+          <t xml:space="preserve">mapping</t>
         </is>
       </c>
       <c r="C74" s="0" t="b">
@@ -5577,7 +5817,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi</t>
+          <t xml:space="preserve">RnD||Membuat</t>
         </is>
       </c>
     </row>
@@ -5589,7 +5829,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">materi</t>
+          <t xml:space="preserve">prompt</t>
         </is>
       </c>
       <c r="C75" s="0" t="b">
@@ -5597,19 +5837,19 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi||Menyusun</t>
+          <t xml:space="preserve">RnD||Membuat</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">journey</t>
+          <t xml:space="preserve">Melakukan</t>
         </is>
       </c>
       <c r="C76" s="0" t="b">
@@ -5617,19 +5857,19 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi||Menyusun</t>
+          <t xml:space="preserve">RnD</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mengambil (take)</t>
+          <t xml:space="preserve">riset</t>
         </is>
       </c>
       <c r="C77" s="0" t="b">
@@ -5637,19 +5877,19 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi</t>
+          <t xml:space="preserve">RnD||Melakukan</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">video pembahasan</t>
+          <t xml:space="preserve">Menyusun</t>
         </is>
       </c>
       <c r="C78" s="0" t="b">
@@ -5657,19 +5897,19 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi||Mengambil (take)</t>
+          <t xml:space="preserve">Develop Materi</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Melakukan</t>
+          <t xml:space="preserve">materi</t>
         </is>
       </c>
       <c r="C79" s="0" t="b">
@@ -5677,7 +5917,7 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi</t>
+          <t xml:space="preserve">Develop Materi||Menyusun</t>
         </is>
       </c>
     </row>
@@ -5689,7 +5929,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">syuting</t>
+          <t xml:space="preserve">journey</t>
         </is>
       </c>
       <c r="C80" s="0" t="b">
@@ -5697,19 +5937,19 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi||Melakukan</t>
+          <t xml:space="preserve">Develop Materi||Menyusun</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">retake</t>
+          <t xml:space="preserve">Mengambil (take)</t>
         </is>
       </c>
       <c r="C81" s="0" t="b">
@@ -5717,19 +5957,19 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Materi||Melakukan</t>
+          <t xml:space="preserve">Develop Materi</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membuat</t>
+          <t xml:space="preserve">video pembahasan</t>
         </is>
       </c>
       <c r="C82" s="0" t="b">
@@ -5737,19 +5977,19 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Soal</t>
+          <t xml:space="preserve">Develop Materi||Mengambil (take)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">soal</t>
+          <t xml:space="preserve">Melakukan</t>
         </is>
       </c>
       <c r="C83" s="0" t="b">
@@ -5757,7 +5997,7 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Soal||Membuat</t>
+          <t xml:space="preserve">Develop Materi</t>
         </is>
       </c>
     </row>
@@ -5769,7 +6009,7 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">pembahasan</t>
+          <t xml:space="preserve">syuting</t>
         </is>
       </c>
       <c r="C84" s="0" t="b">
@@ -5777,19 +6017,19 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Soal||Membuat</t>
+          <t xml:space="preserve">Develop Materi||Melakukan</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menyusun</t>
+          <t xml:space="preserve">retake</t>
         </is>
       </c>
       <c r="C85" s="0" t="b">
@@ -5797,19 +6037,19 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Soal</t>
+          <t xml:space="preserve">Develop Materi||Melakukan</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">paket tryout</t>
+          <t xml:space="preserve">Membuat</t>
         </is>
       </c>
       <c r="C86" s="0" t="b">
@@ -5817,19 +6057,19 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop Soal||Menyusun</t>
+          <t xml:space="preserve">Develop Soal</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Melakukan</t>
+          <t xml:space="preserve">soal</t>
         </is>
       </c>
       <c r="C87" s="0" t="b">
@@ -5837,7 +6077,7 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">QC Konten</t>
+          <t xml:space="preserve">Develop Soal||Membuat</t>
         </is>
       </c>
     </row>
@@ -5849,7 +6089,7 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">QC</t>
+          <t xml:space="preserve">pembahasan</t>
         </is>
       </c>
       <c r="C88" s="0" t="b">
@@ -5857,7 +6097,7 @@
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">QC Konten||Melakukan</t>
+          <t xml:space="preserve">Develop Soal||Membuat</t>
         </is>
       </c>
     </row>
@@ -5869,7 +6109,7 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Memperbarui</t>
+          <t xml:space="preserve">Menyusun</t>
         </is>
       </c>
       <c r="C89" s="0" t="b">
@@ -5877,7 +6117,7 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">QC Konten</t>
+          <t xml:space="preserve">Develop Soal</t>
         </is>
       </c>
     </row>
@@ -5889,7 +6129,7 @@
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bumper</t>
+          <t xml:space="preserve">paket tryout</t>
         </is>
       </c>
       <c r="C90" s="0" t="b">
@@ -5897,19 +6137,19 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">QC Konten||Memperbarui</t>
+          <t xml:space="preserve">Develop Soal||Menyusun</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">thumbnail</t>
+          <t xml:space="preserve">Melakukan</t>
         </is>
       </c>
       <c r="C91" s="0" t="b">
@@ -5917,19 +6157,19 @@
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">QC Konten||Memperbarui</t>
+          <t xml:space="preserve">QC Konten</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menginput</t>
+          <t xml:space="preserve">QC</t>
         </is>
       </c>
       <c r="C92" s="0" t="b">
@@ -5937,19 +6177,19 @@
       </c>
       <c r="D92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Input</t>
+          <t xml:space="preserve">QC Konten||Melakukan</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">soal</t>
+          <t xml:space="preserve">Memperbarui</t>
         </is>
       </c>
       <c r="C93" s="0" t="b">
@@ -5957,7 +6197,7 @@
       </c>
       <c r="D93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Input||Menginput</t>
+          <t xml:space="preserve">QC Konten</t>
         </is>
       </c>
     </row>
@@ -5969,7 +6209,7 @@
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">video pembahasan</t>
+          <t xml:space="preserve">bumper</t>
         </is>
       </c>
       <c r="C94" s="0" t="b">
@@ -5977,7 +6217,7 @@
       </c>
       <c r="D94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Input||Menginput</t>
+          <t xml:space="preserve">QC Konten||Memperbarui</t>
         </is>
       </c>
     </row>
@@ -5989,7 +6229,7 @@
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">jadwal</t>
+          <t xml:space="preserve">thumbnail</t>
         </is>
       </c>
       <c r="C95" s="0" t="b">
@@ -5997,7 +6237,7 @@
       </c>
       <c r="D95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Input||Menginput</t>
+          <t xml:space="preserve">QC Konten||Memperbarui</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6249,7 @@
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membangun</t>
+          <t xml:space="preserve">Menginput</t>
         </is>
       </c>
       <c r="C96" s="0" t="b">
@@ -6029,7 +6269,7 @@
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">sistem otomatis</t>
+          <t xml:space="preserve">soal</t>
         </is>
       </c>
       <c r="C97" s="0" t="b">
@@ -6037,19 +6277,19 @@
       </c>
       <c r="D97" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Input||Membangun</t>
+          <t xml:space="preserve">Input||Menginput</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Memonitor</t>
+          <t xml:space="preserve">video pembahasan</t>
         </is>
       </c>
       <c r="C98" s="0" t="b">
@@ -6057,7 +6297,7 @@
       </c>
       <c r="D98" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liveclass</t>
+          <t xml:space="preserve">Input||Menginput</t>
         </is>
       </c>
     </row>
@@ -6069,7 +6309,7 @@
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">liveclass</t>
+          <t xml:space="preserve">jadwal</t>
         </is>
       </c>
       <c r="C99" s="0" t="b">
@@ -6077,7 +6317,7 @@
       </c>
       <c r="D99" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liveclass||Memonitor</t>
+          <t xml:space="preserve">Input||Menginput</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6329,7 @@
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menyusun</t>
+          <t xml:space="preserve">Membangun</t>
         </is>
       </c>
       <c r="C100" s="0" t="b">
@@ -6097,7 +6337,7 @@
       </c>
       <c r="D100" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liveclass</t>
+          <t xml:space="preserve">Input</t>
         </is>
       </c>
     </row>
@@ -6109,7 +6349,7 @@
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">jadwal</t>
+          <t xml:space="preserve">sistem otomatis</t>
         </is>
       </c>
       <c r="C101" s="0" t="b">
@@ -6117,7 +6357,7 @@
       </c>
       <c r="D101" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liveclass||Menyusun</t>
+          <t xml:space="preserve">Input||Membangun</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6369,7 @@
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Merapikan</t>
+          <t xml:space="preserve">Memonitor</t>
         </is>
       </c>
       <c r="C102" s="0" t="b">
@@ -6137,7 +6377,7 @@
       </c>
       <c r="D102" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Sistem</t>
+          <t xml:space="preserve">Liveclass</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6389,7 @@
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">subbab</t>
+          <t xml:space="preserve">liveclass</t>
         </is>
       </c>
       <c r="C103" s="0" t="b">
@@ -6157,7 +6397,7 @@
       </c>
       <c r="D103" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Sistem||Merapikan</t>
+          <t xml:space="preserve">Liveclass||Memonitor</t>
         </is>
       </c>
     </row>
@@ -6177,7 +6417,7 @@
       </c>
       <c r="D104" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Sistem</t>
+          <t xml:space="preserve">Liveclass</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6429,7 @@
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">kerangka kategori</t>
+          <t xml:space="preserve">jadwal</t>
         </is>
       </c>
       <c r="C105" s="0" t="b">
@@ -6197,7 +6437,7 @@
       </c>
       <c r="D105" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Sistem||Menyusun</t>
+          <t xml:space="preserve">Liveclass||Menyusun</t>
         </is>
       </c>
     </row>
@@ -6209,7 +6449,7 @@
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generate/regenerate</t>
+          <t xml:space="preserve">Merapikan</t>
         </is>
       </c>
       <c r="C106" s="0" t="b">
@@ -6229,7 +6469,7 @@
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">paket</t>
+          <t xml:space="preserve">subbab</t>
         </is>
       </c>
       <c r="C107" s="0" t="b">
@@ -6237,7 +6477,7 @@
       </c>
       <c r="D107" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Sistem||Generate/regenerate</t>
+          <t xml:space="preserve">Manajemen Sistem||Merapikan</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6489,7 @@
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menampilkan/menyembunyikan</t>
+          <t xml:space="preserve">Menyusun</t>
         </is>
       </c>
       <c r="C108" s="0" t="b">
@@ -6269,7 +6509,7 @@
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">kategori</t>
+          <t xml:space="preserve">kerangka kategori</t>
         </is>
       </c>
       <c r="C109" s="0" t="b">
@@ -6277,7 +6517,7 @@
       </c>
       <c r="D109" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Sistem||Menampilkan/menyembunyikan</t>
+          <t xml:space="preserve">Manajemen Sistem||Menyusun</t>
         </is>
       </c>
     </row>
@@ -6289,7 +6529,7 @@
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mendistribusikan</t>
+          <t xml:space="preserve">Generate/regenerate</t>
         </is>
       </c>
       <c r="C110" s="0" t="b">
@@ -6297,7 +6537,7 @@
       </c>
       <c r="D110" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Guru</t>
+          <t xml:space="preserve">Manajemen Sistem</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6549,7 @@
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">proyek video pembahasan</t>
+          <t xml:space="preserve">paket</t>
         </is>
       </c>
       <c r="C111" s="0" t="b">
@@ -6317,19 +6557,19 @@
       </c>
       <c r="D111" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Guru||Mendistribusikan</t>
+          <t xml:space="preserve">Manajemen Sistem||Generate/regenerate</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">proyek komplit</t>
+          <t xml:space="preserve">Menampilkan/menyembunyikan</t>
         </is>
       </c>
       <c r="C112" s="0" t="b">
@@ -6337,19 +6577,19 @@
       </c>
       <c r="D112" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Guru||Mendistribusikan</t>
+          <t xml:space="preserve">Manajemen Sistem</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B113" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menyusun</t>
+          <t xml:space="preserve">kategori</t>
         </is>
       </c>
       <c r="C113" s="0" t="b">
@@ -6357,19 +6597,19 @@
       </c>
       <c r="D113" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Guru</t>
+          <t xml:space="preserve">Manajemen Sistem||Menampilkan/menyembunyikan</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">verb</t>
         </is>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">jadwal</t>
+          <t xml:space="preserve">Mendistribusikan</t>
         </is>
       </c>
       <c r="C114" s="0" t="b">
@@ -6377,19 +6617,19 @@
       </c>
       <c r="D114" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manajemen Guru||Menyusun</t>
+          <t xml:space="preserve">Manajemen Guru</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">verb</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membuat</t>
+          <t xml:space="preserve">proyek video pembahasan</t>
         </is>
       </c>
       <c r="C115" s="0" t="b">
@@ -6397,7 +6637,7 @@
       </c>
       <c r="D115" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data &amp; Intelligence</t>
+          <t xml:space="preserve">Manajemen Guru||Mendistribusikan</t>
         </is>
       </c>
     </row>
@@ -6409,7 +6649,7 @@
       </c>
       <c r="B116" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">query</t>
+          <t xml:space="preserve">proyek komplit</t>
         </is>
       </c>
       <c r="C116" s="0" t="b">
@@ -6417,7 +6657,7 @@
       </c>
       <c r="D116" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data &amp; Intelligence||Membuat</t>
+          <t xml:space="preserve">Manajemen Guru||Mendistribusikan</t>
         </is>
       </c>
     </row>
@@ -6429,7 +6669,7 @@
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Melakukan</t>
+          <t xml:space="preserve">Menyusun</t>
         </is>
       </c>
       <c r="C117" s="0" t="b">
@@ -6437,7 +6677,7 @@
       </c>
       <c r="D117" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data &amp; Intelligence</t>
+          <t xml:space="preserve">Manajemen Guru</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6689,7 @@
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scraping</t>
+          <t xml:space="preserve">jadwal</t>
         </is>
       </c>
       <c r="C118" s="0" t="b">
@@ -6457,7 +6697,7 @@
       </c>
       <c r="D118" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data &amp; Intelligence||Melakukan</t>
+          <t xml:space="preserve">Manajemen Guru||Menyusun</t>
         </is>
       </c>
     </row>
@@ -6469,7 +6709,7 @@
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membangun</t>
+          <t xml:space="preserve">Membuat</t>
         </is>
       </c>
       <c r="C119" s="0" t="b">
@@ -6489,7 +6729,7 @@
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">dashboard</t>
+          <t xml:space="preserve">query</t>
         </is>
       </c>
       <c r="C120" s="0" t="b">
@@ -6497,7 +6737,7 @@
       </c>
       <c r="D120" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data &amp; Intelligence||Membangun</t>
+          <t xml:space="preserve">Data &amp; Intelligence||Membuat</t>
         </is>
       </c>
     </row>
@@ -6509,7 +6749,7 @@
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Menyelesaikan</t>
+          <t xml:space="preserve">Melakukan</t>
         </is>
       </c>
       <c r="C121" s="0" t="b">
@@ -6517,7 +6757,7 @@
       </c>
       <c r="D121" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report</t>
+          <t xml:space="preserve">Data &amp; Intelligence</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6769,7 @@
       </c>
       <c r="B122" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">scraping</t>
         </is>
       </c>
       <c r="C122" s="0" t="b">
@@ -6537,7 +6777,7 @@
       </c>
       <c r="D122" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report||Menyelesaikan</t>
+          <t xml:space="preserve">Data &amp; Intelligence||Melakukan</t>
         </is>
       </c>
     </row>
@@ -6549,7 +6789,7 @@
       </c>
       <c r="B123" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mengelompokkan</t>
+          <t xml:space="preserve">Membangun</t>
         </is>
       </c>
       <c r="C123" s="0" t="b">
@@ -6557,7 +6797,7 @@
       </c>
       <c r="D123" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report</t>
+          <t xml:space="preserve">Data &amp; Intelligence</t>
         </is>
       </c>
     </row>
@@ -6569,13 +6809,93 @@
       </c>
       <c r="B124" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">dashboard</t>
+        </is>
+      </c>
+      <c r="C124" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="D124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data &amp; Intelligence||Membangun</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verb</t>
+        </is>
+      </c>
+      <c r="B125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Menyelesaikan</t>
+        </is>
+      </c>
+      <c r="C125" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="D125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">object</t>
+        </is>
+      </c>
+      <c r="B126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
+        </is>
+      </c>
+      <c r="C126" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="D126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Report||Menyelesaikan</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verb</t>
+        </is>
+      </c>
+      <c r="B127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mengelompokkan</t>
+        </is>
+      </c>
+      <c r="C127" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="D127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">object</t>
+        </is>
+      </c>
+      <c r="B128" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">data</t>
         </is>
       </c>
-      <c r="C124" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="D124" s="0" t="inlineStr">
+      <c r="C128" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="D128" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Report||Mengelompokkan</t>
         </is>
@@ -6618,7 +6938,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>46224.385416666664</v>
+        <v>46225.385416666664</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
@@ -6638,7 +6958,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>46224.41805555556</v>
+        <v>46225.41805555556</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
@@ -6658,7 +6978,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>46225.36111111111</v>
+        <v>46226.36111111111</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
@@ -6678,7 +6998,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>46227.555555555555</v>
+        <v>46228.555555555555</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
@@ -6698,7 +7018,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>46228.37847222222</v>
+        <v>46229.37847222222</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
@@ -6718,7 +7038,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>46229.479166666664</v>
+        <v>46230.479166666664</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
@@ -6738,7 +7058,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>46229.59027777778</v>
+        <v>46230.59027777778</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
@@ -6758,7 +7078,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>46230.447916666664</v>
+        <v>46231.447916666664</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
@@ -6778,7 +7098,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>46230.625</v>
+        <v>46231.625</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
@@ -6798,7 +7118,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <v>46231.395833333336</v>
+        <v>46232.395833333336</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
@@ -6818,7 +7138,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2">
-        <v>46231.680555555555</v>
+        <v>46232.680555555555</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
@@ -6838,7 +7158,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2">
-        <v>46232.37152777778</v>
+        <v>46233.37152777778</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
@@ -6858,7 +7178,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <v>46232.569444444445</v>
+        <v>46233.569444444445</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
@@ -6878,7 +7198,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2">
-        <v>46232.600694444445</v>
+        <v>46233.600694444445</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
@@ -6898,7 +7218,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2">
-        <v>46233.381944444445</v>
+        <v>46234.381944444445</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
@@ -6918,7 +7238,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2">
-        <v>46228.416666666664</v>
+        <v>46229.416666666664</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
@@ -6938,7 +7258,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2">
-        <v>46229.46875</v>
+        <v>46230.46875</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
@@ -6958,7 +7278,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2">
-        <v>46226.40625</v>
+        <v>46227.40625</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
@@ -6978,7 +7298,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2">
-        <v>46231.4375</v>
+        <v>46232.4375</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
@@ -6998,7 +7318,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2">
-        <v>46227.65972222222</v>
+        <v>46228.65972222222</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
@@ -7088,7 +7408,7 @@
         </is>
       </c>
       <c r="F2" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="3">
@@ -7116,7 +7436,7 @@
         </is>
       </c>
       <c r="F3" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="4">
@@ -7144,7 +7464,7 @@
         </is>
       </c>
       <c r="F4" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="5">
@@ -7232,7 +7552,7 @@
         </is>
       </c>
       <c r="F8" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="9">
@@ -7260,7 +7580,7 @@
         </is>
       </c>
       <c r="F9" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="10">
@@ -7288,7 +7608,7 @@
         </is>
       </c>
       <c r="F10" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="11">
@@ -7316,7 +7636,7 @@
         </is>
       </c>
       <c r="F11" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="12">
@@ -7364,7 +7684,7 @@
         </is>
       </c>
       <c r="F13" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="14">
@@ -7392,7 +7712,7 @@
         </is>
       </c>
       <c r="F14" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="15">
@@ -7460,7 +7780,7 @@
         </is>
       </c>
       <c r="F17" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="18">
@@ -7648,7 +7968,7 @@
         </is>
       </c>
       <c r="F26" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="27">
@@ -7676,7 +7996,7 @@
         </is>
       </c>
       <c r="F27" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="28">
@@ -7704,7 +8024,7 @@
         </is>
       </c>
       <c r="F28" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="29">
@@ -7732,7 +8052,7 @@
         </is>
       </c>
       <c r="F29" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="30">
@@ -7760,7 +8080,7 @@
         </is>
       </c>
       <c r="F30" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="31">
@@ -7788,7 +8108,7 @@
         </is>
       </c>
       <c r="F31" s="2">
-        <v>46230.416666666664</v>
+        <v>46231.416666666664</v>
       </c>
     </row>
     <row r="32">
@@ -7856,7 +8176,7 @@
         </is>
       </c>
       <c r="F34" s="2">
-        <v>46231.458333333336</v>
+        <v>46232.458333333336</v>
       </c>
     </row>
     <row r="35">
@@ -7884,7 +8204,7 @@
         </is>
       </c>
       <c r="F35" s="2">
-        <v>46231.458333333336</v>
+        <v>46232.458333333336</v>
       </c>
     </row>
     <row r="36">
@@ -7972,7 +8292,7 @@
         </is>
       </c>
       <c r="F39" s="2">
-        <v>46231.458333333336</v>
+        <v>46232.458333333336</v>
       </c>
     </row>
     <row r="40">
@@ -8000,7 +8320,7 @@
         </is>
       </c>
       <c r="F40" s="2">
-        <v>46231.458333333336</v>
+        <v>46232.458333333336</v>
       </c>
     </row>
     <row r="41">
@@ -8028,7 +8348,7 @@
         </is>
       </c>
       <c r="F41" s="2">
-        <v>46231.458333333336</v>
+        <v>46232.458333333336</v>
       </c>
     </row>
     <row r="42">
@@ -8056,7 +8376,7 @@
         </is>
       </c>
       <c r="F42" s="2">
-        <v>46231.458333333336</v>
+        <v>46232.458333333336</v>
       </c>
     </row>
     <row r="43">
@@ -8084,7 +8404,7 @@
         </is>
       </c>
       <c r="F43" s="2">
-        <v>46231.458333333336</v>
+        <v>46232.458333333336</v>
       </c>
     </row>
     <row r="44">
@@ -8299,10 +8619,10 @@
         </is>
       </c>
       <c r="F2" s="2">
-        <v>46203.375</v>
+        <v>46204.375</v>
       </c>
       <c r="G2" s="1">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="H2" s="0" t="inlineStr">
         <is>
@@ -8342,10 +8662,10 @@
         </is>
       </c>
       <c r="F3" s="2">
-        <v>46188.375</v>
+        <v>46189.375</v>
       </c>
       <c r="G3" s="1">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
@@ -8385,10 +8705,10 @@
         </is>
       </c>
       <c r="F4" s="2">
-        <v>46193.375</v>
+        <v>46194.375</v>
       </c>
       <c r="G4" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
@@ -8428,10 +8748,10 @@
         </is>
       </c>
       <c r="F5" s="2">
-        <v>46219.375</v>
+        <v>46220.375</v>
       </c>
       <c r="G5" s="1">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
@@ -8471,10 +8791,10 @@
         </is>
       </c>
       <c r="F6" s="2">
-        <v>46225.375</v>
+        <v>46226.375</v>
       </c>
       <c r="G6" s="1">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
@@ -8509,10 +8829,10 @@
         </is>
       </c>
       <c r="F7" s="2">
-        <v>46223.375</v>
+        <v>46224.375</v>
       </c>
       <c r="G7" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
@@ -8605,7 +8925,7 @@
         </is>
       </c>
       <c r="E2" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="F2" s="0" t="b">
         <v>1</v>
@@ -8616,7 +8936,7 @@
         </is>
       </c>
       <c r="H2" s="2">
-        <v>46228.666666666664</v>
+        <v>46229.666666666664</v>
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
@@ -8644,7 +8964,7 @@
         </is>
       </c>
       <c r="E3" s="1">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="F3" s="0" t="b">
         <v>0</v>
@@ -8675,7 +8995,7 @@
         </is>
       </c>
       <c r="E4" s="1">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="F4" s="0" t="b">
         <v>0</v>
@@ -8701,7 +9021,7 @@
         </is>
       </c>
       <c r="E5" s="1">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F5" s="0" t="b">
         <v>0</v>
@@ -8727,7 +9047,7 @@
         </is>
       </c>
       <c r="E6" s="1">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F6" s="0" t="b">
         <v>0</v>
@@ -8753,7 +9073,7 @@
         </is>
       </c>
       <c r="E7" s="1">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="F7" s="0" t="b">
         <v>1</v>
@@ -8764,7 +9084,7 @@
         </is>
       </c>
       <c r="H7" s="2">
-        <v>46214.666666666664</v>
+        <v>46215.666666666664</v>
       </c>
     </row>
     <row r="8">
@@ -8787,7 +9107,7 @@
         </is>
       </c>
       <c r="E8" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="F8" s="0" t="b">
         <v>1</v>
@@ -8798,7 +9118,7 @@
         </is>
       </c>
       <c r="H8" s="2">
-        <v>46224.666666666664</v>
+        <v>46225.666666666664</v>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
@@ -8826,7 +9146,7 @@
         </is>
       </c>
       <c r="E9" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F9" s="0" t="b">
         <v>1</v>
@@ -8837,7 +9157,7 @@
         </is>
       </c>
       <c r="H9" s="2">
-        <v>46232.666666666664</v>
+        <v>46233.666666666664</v>
       </c>
     </row>
     <row r="10">
@@ -8860,7 +9180,7 @@
         </is>
       </c>
       <c r="E10" s="1">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="F10" s="0" t="b">
         <v>0</v>
@@ -8886,7 +9206,7 @@
         </is>
       </c>
       <c r="E11" s="1">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="F11" s="0" t="b">
         <v>0</v>
@@ -8912,7 +9232,7 @@
         </is>
       </c>
       <c r="E12" s="1">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="F12" s="0" t="b">
         <v>0</v>
@@ -8938,7 +9258,7 @@
         </is>
       </c>
       <c r="E13" s="1">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="F13" s="0" t="b">
         <v>1</v>
@@ -8949,7 +9269,7 @@
         </is>
       </c>
       <c r="H13" s="2">
-        <v>46209.666666666664</v>
+        <v>46210.666666666664</v>
       </c>
     </row>
     <row r="14">
@@ -8972,7 +9292,7 @@
         </is>
       </c>
       <c r="E14" s="1">
-        <v>46215</v>
+        <v>46216</v>
       </c>
       <c r="F14" s="0" t="b">
         <v>1</v>
@@ -8983,7 +9303,7 @@
         </is>
       </c>
       <c r="H14" s="2">
-        <v>46216.666666666664</v>
+        <v>46217.666666666664</v>
       </c>
     </row>
     <row r="15">
@@ -9006,7 +9326,7 @@
         </is>
       </c>
       <c r="E15" s="1">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="F15" s="0" t="b">
         <v>1</v>
@@ -9017,7 +9337,7 @@
         </is>
       </c>
       <c r="H15" s="2">
-        <v>46226.666666666664</v>
+        <v>46227.666666666664</v>
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
@@ -9045,7 +9365,7 @@
         </is>
       </c>
       <c r="E16" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="F16" s="0" t="b">
         <v>1</v>
@@ -9056,7 +9376,7 @@
         </is>
       </c>
       <c r="H16" s="2">
-        <v>46231.666666666664</v>
+        <v>46232.666666666664</v>
       </c>
     </row>
     <row r="17">
@@ -9079,7 +9399,7 @@
         </is>
       </c>
       <c r="E17" s="1">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F17" s="0" t="b">
         <v>1</v>
@@ -9090,7 +9410,7 @@
         </is>
       </c>
       <c r="H17" s="2">
-        <v>46233.666666666664</v>
+        <v>46234.666666666664</v>
       </c>
     </row>
     <row r="18">
@@ -9113,7 +9433,7 @@
         </is>
       </c>
       <c r="E18" s="1">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F18" s="0" t="b">
         <v>0</v>
@@ -9139,7 +9459,7 @@
         </is>
       </c>
       <c r="E19" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F19" s="0" t="b">
         <v>0</v>
@@ -9165,7 +9485,7 @@
         </is>
       </c>
       <c r="E20" s="1">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="F20" s="0" t="b">
         <v>0</v>
@@ -9191,7 +9511,7 @@
         </is>
       </c>
       <c r="E21" s="1">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="F21" s="0" t="b">
         <v>0</v>
@@ -9217,7 +9537,7 @@
         </is>
       </c>
       <c r="E22" s="1">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="F22" s="0" t="b">
         <v>0</v>
@@ -9243,7 +9563,7 @@
         </is>
       </c>
       <c r="E23" s="1">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F23" s="0" t="b">
         <v>0</v>
@@ -9269,7 +9589,7 @@
         </is>
       </c>
       <c r="E24" s="1">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="F24" s="0" t="b">
         <v>0</v>
@@ -9295,7 +9615,7 @@
         </is>
       </c>
       <c r="E25" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="F25" s="0" t="b">
         <v>1</v>
@@ -9306,7 +9626,7 @@
         </is>
       </c>
       <c r="H25" s="2">
-        <v>46233.666666666664</v>
+        <v>46234.666666666664</v>
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
@@ -9334,7 +9654,7 @@
         </is>
       </c>
       <c r="E26" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="F26" s="0" t="b">
         <v>0</v>
@@ -9360,7 +9680,7 @@
         </is>
       </c>
       <c r="E27" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F27" s="0" t="b">
         <v>0</v>
@@ -9457,7 +9777,7 @@
         </is>
       </c>
       <c r="G2" s="2">
-        <v>46226.583333333336</v>
+        <v>46227.583333333336</v>
       </c>
       <c r="H2" s="0" t="b">
         <v>0</v>
@@ -9495,7 +9815,7 @@
         </is>
       </c>
       <c r="G3" s="2">
-        <v>46229.708333333336</v>
+        <v>46230.708333333336</v>
       </c>
       <c r="H3" s="0" t="b">
         <v>0</v>
@@ -9533,7 +9853,7 @@
         </is>
       </c>
       <c r="G4" s="2">
-        <v>46229.59027777778</v>
+        <v>46230.59027777778</v>
       </c>
       <c r="H4" s="0" t="b">
         <v>0</v>
@@ -9571,7 +9891,7 @@
         </is>
       </c>
       <c r="G5" s="2">
-        <v>46230.447916666664</v>
+        <v>46231.447916666664</v>
       </c>
       <c r="H5" s="0" t="b">
         <v>1</v>
@@ -9609,7 +9929,7 @@
         </is>
       </c>
       <c r="G6" s="2">
-        <v>46231.680555555555</v>
+        <v>46232.680555555555</v>
       </c>
       <c r="H6" s="0" t="b">
         <v>1</v>
@@ -9647,7 +9967,7 @@
         </is>
       </c>
       <c r="G7" s="2">
-        <v>46228.37847222222</v>
+        <v>46229.37847222222</v>
       </c>
       <c r="H7" s="0" t="b">
         <v>0</v>
@@ -9685,7 +10005,7 @@
         </is>
       </c>
       <c r="G8" s="2">
-        <v>46228.37847222222</v>
+        <v>46229.37847222222</v>
       </c>
       <c r="H8" s="0" t="b">
         <v>0</v>
@@ -9723,7 +10043,7 @@
         </is>
       </c>
       <c r="G9" s="2">
-        <v>46232.569444444445</v>
+        <v>46233.569444444445</v>
       </c>
       <c r="H9" s="0" t="b">
         <v>0</v>
@@ -9761,7 +10081,7 @@
         </is>
       </c>
       <c r="G10" s="2">
-        <v>46229.46875</v>
+        <v>46230.46875</v>
       </c>
       <c r="H10" s="0" t="b">
         <v>0</v>
@@ -9810,7 +10130,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>46219.375</v>
+        <v>46220.375</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
@@ -9835,7 +10155,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>46221.427083333336</v>
+        <v>46222.427083333336</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
@@ -9860,7 +10180,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>46223.354166666664</v>
+        <v>46224.354166666664</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
@@ -9885,7 +10205,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>46224.385416666664</v>
+        <v>46225.385416666664</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
@@ -9910,7 +10230,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>46224.41805555556</v>
+        <v>46225.41805555556</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
@@ -9935,7 +10255,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>46225.458333333336</v>
+        <v>46226.458333333336</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
@@ -9960,7 +10280,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>46225.479166666664</v>
+        <v>46226.479166666664</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
@@ -9985,7 +10305,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>46226.40625</v>
+        <v>46227.40625</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
@@ -10010,7 +10330,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>46226.583333333336</v>
+        <v>46227.583333333336</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
@@ -10035,7 +10355,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <v>46227.555555555555</v>
+        <v>46228.555555555555</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
@@ -10060,7 +10380,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2">
-        <v>46227.65972222222</v>
+        <v>46228.65972222222</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
@@ -10085,7 +10405,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2">
-        <v>46228.37847222222</v>
+        <v>46229.37847222222</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
@@ -10110,7 +10430,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <v>46228.416666666664</v>
+        <v>46229.416666666664</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
@@ -10135,7 +10455,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2">
-        <v>46228.6875</v>
+        <v>46229.6875</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
@@ -10160,7 +10480,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2">
-        <v>46229.46875</v>
+        <v>46230.46875</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
@@ -10185,7 +10505,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2">
-        <v>46229.479166666664</v>
+        <v>46230.479166666664</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
@@ -10210,7 +10530,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2">
-        <v>46229.59027777778</v>
+        <v>46230.59027777778</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
@@ -10235,7 +10555,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2">
-        <v>46229.708333333336</v>
+        <v>46230.708333333336</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
@@ -10260,7 +10580,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2">
-        <v>46230.447916666664</v>
+        <v>46231.447916666664</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
@@ -10285,7 +10605,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2">
-        <v>46230.625</v>
+        <v>46231.625</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
@@ -10310,7 +10630,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2">
-        <v>46230.67361111111</v>
+        <v>46231.67361111111</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
@@ -10335,7 +10655,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2">
-        <v>46231.395833333336</v>
+        <v>46232.395833333336</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
@@ -10360,7 +10680,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2">
-        <v>46231.4375</v>
+        <v>46232.4375</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
@@ -10385,7 +10705,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2">
-        <v>46231.541666666664</v>
+        <v>46232.541666666664</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
@@ -10410,7 +10730,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2">
-        <v>46231.680555555555</v>
+        <v>46232.680555555555</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
@@ -10435,7 +10755,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2">
-        <v>46232.37152777778</v>
+        <v>46233.37152777778</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
@@ -10460,7 +10780,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2">
-        <v>46232.395833333336</v>
+        <v>46233.395833333336</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
@@ -10485,7 +10805,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2">
-        <v>46232.569444444445</v>
+        <v>46233.569444444445</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
@@ -10510,7 +10830,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2">
-        <v>46232.600694444445</v>
+        <v>46233.600694444445</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
@@ -10535,7 +10855,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2">
-        <v>46232.645833333336</v>
+        <v>46233.645833333336</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
@@ -10560,7 +10880,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <v>46233.34375</v>
+        <v>46234.34375</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
@@ -10585,7 +10905,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2">
-        <v>46233.381944444445</v>
+        <v>46234.381944444445</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
@@ -10610,7 +10930,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2">
-        <v>46233.40277777778</v>
+        <v>46234.40277777778</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
@@ -10635,7 +10955,7 @@
     </row>
     <row r="35">
       <c r="A35" s="2">
-        <v>46233.430555555555</v>
+        <v>46234.430555555555</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
@@ -10825,15 +11145,45 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Magang Konten</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magang</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magang Data</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magang</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Lintas Divisi</t>
         </is>
       </c>
-      <c r="B11" s="0" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Lihat Saja</t>
         </is>
       </c>
-      <c r="C11" s="0" t="b">
+      <c r="C13" s="0" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>